<commit_message>
Restore resources link column
</commit_message>
<xml_diff>
--- a/public/example-files/import_resources_en.xlsx
+++ b/public/example-files/import_resources_en.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
   <si>
     <t>Category</t>
   </si>
@@ -68,6 +68,9 @@
   </si>
   <si>
     <t>Access Requirements</t>
+  </si>
+  <si>
+    <t>Link</t>
   </si>
 </sst>
 </file>
@@ -329,13 +332,13 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="8" max="8" width="28.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -363,8 +366,11 @@
       <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J1" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -387,8 +393,9 @@
       <c r="I2" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J2" s="1"/>
+    </row>
+    <row r="3" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -400,8 +407,9 @@
         <v>14</v>
       </c>
       <c r="I3" s="1"/>
-    </row>
-    <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J3" s="1"/>
+    </row>
+    <row r="4" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -412,8 +420,9 @@
         <v>14</v>
       </c>
       <c r="I4" s="1"/>
-    </row>
-    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J4" s="1"/>
+    </row>
+    <row r="5" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -424,8 +433,9 @@
         <v>14</v>
       </c>
       <c r="I5" s="1"/>
-    </row>
-    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J5" s="1"/>
+    </row>
+    <row r="6" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -437,6 +447,7 @@
         <v>14</v>
       </c>
       <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>